<commit_message>
Refining Companion UI: Center Logo, Full-Screen Filigree Background, and Production-Ready Voice Wave Visualizer with Dynamic Frequency Pulse
</commit_message>
<xml_diff>
--- a/backend/EpicVerse_New_Invites.xlsx
+++ b/backend/EpicVerse_New_Invites.xlsx
@@ -426,3500 +426,3500 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>8Q8CTV</t>
+          <t>TNXN1C</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>VUR418</t>
+          <t>EXQN0K</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DI1VWS</t>
+          <t>65KMGE</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>E0BF76</t>
+          <t>ZVZTDB</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MD44SH</t>
+          <t>I2DZR6</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>11260L</t>
+          <t>QP8EHA</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>58JOZH</t>
+          <t>PBZ3BQ</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ZIJG1C</t>
+          <t>U4DNSZ</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>R5N16H</t>
+          <t>WK2WHC</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>FALWYT</t>
+          <t>3JHRIF</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ZJCFNF</t>
+          <t>6BRPDE</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>82837B</t>
+          <t>QV9JD0</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>4X45Y6</t>
+          <t>T9DEJZ</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>DVY7SK</t>
+          <t>M5VS56</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>G8H3XQ</t>
+          <t>TD8KRA</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>6D072P</t>
+          <t>P6AU5F</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0IDWYA</t>
+          <t>95SG1E</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CSZP7A</t>
+          <t>1MF5V3</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>3DUOI4</t>
+          <t>V18R2I</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TTY73P</t>
+          <t>MJ8RAX</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>HEP0HN</t>
+          <t>05WWQM</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SZMION</t>
+          <t>JWEIOT</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>G52YNW</t>
+          <t>AC7EFE</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>I79SMO</t>
+          <t>D0RX93</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ZZ2IDU</t>
+          <t>VQ0SI7</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>GEK33G</t>
+          <t>EW3IIX</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>OF86HC</t>
+          <t>Q1UZLV</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>BUI88Y</t>
+          <t>XI4B4K</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>DPN2JN</t>
+          <t>ZMXHIK</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>RLM6O9</t>
+          <t>ISMLZE</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>5ES783</t>
+          <t>XHYN2C</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>DAX0Q8</t>
+          <t>W1U3JN</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>JW3OYJ</t>
+          <t>3GCRIH</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>88S2M9</t>
+          <t>WYCDUE</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>M0I6RP</t>
+          <t>EY74TH</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>TVAXXS</t>
+          <t>FUNPNW</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>9WYV5J</t>
+          <t>4ELPNK</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Q1YX1A</t>
+          <t>I769TL</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>VT3QPH</t>
+          <t>IC8Y5G</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ST2QPM</t>
+          <t>II98GX</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0CWDMX</t>
+          <t>29MK9B</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>I7YX0M</t>
+          <t>422AJJ</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>EUOTHX</t>
+          <t>84KCV7</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>3HSJER</t>
+          <t>V2VUWS</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>OJI3ZC</t>
+          <t>XKIJEZ</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>5GX8F0</t>
+          <t>435MI3</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>V3ACJF</t>
+          <t>O5K1VP</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>XAI4DU</t>
+          <t>HM5YI5</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>QK2V7O</t>
+          <t>WZ0SP5</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>70T6D1</t>
+          <t>8ES1O4</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>23AW55</t>
+          <t>4BOJVM</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>9I0EBF</t>
+          <t>YB1GF5</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>TYZ29Q</t>
+          <t>T4K7OF</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>V4LS81</t>
+          <t>C59TCM</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>7N9LKS</t>
+          <t>2LH5K6</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>OHCLRK</t>
+          <t>WR610R</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>VCY2VE</t>
+          <t>3SN22M</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>M0FUA2</t>
+          <t>RRPDVF</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>FGSSSM</t>
+          <t>B92DBG</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>EX0BBV</t>
+          <t>39JUSS</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>398UFU</t>
+          <t>8FXIQQ</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>IU2FDH</t>
+          <t>61IL1B</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>7MHFX1</t>
+          <t>C6JUZ3</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>AHKTMU</t>
+          <t>RD3J0L</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>TRUAI3</t>
+          <t>C11SYB</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>XTLFU2</t>
+          <t>JFN70E</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2B966S</t>
+          <t>S21PF9</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>JH7Y2Z</t>
+          <t>GF1QHS</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>9LCY3G</t>
+          <t>TMAHF1</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>HHM4C6</t>
+          <t>LM03NM</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>L9QTQ8</t>
+          <t>FGBQRD</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>NI61Q6</t>
+          <t>XK8K5A</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>BYF0PQ</t>
+          <t>9CD0GI</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>YJ5QBQ</t>
+          <t>CRFKOT</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>OXYQ5P</t>
+          <t>YIY3CJ</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>PG44G9</t>
+          <t>TW4X9F</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>9ERHY4</t>
+          <t>P2ZPVO</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>X1MLAL</t>
+          <t>7TI7G3</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>MX1LBO</t>
+          <t>V5VJMZ</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>M2HHK4</t>
+          <t>RVOO25</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Q41XA4</t>
+          <t>KUCCTX</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>LVUREP</t>
+          <t>WROHP8</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>YH4RDL</t>
+          <t>XJLY9S</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>8OMD62</t>
+          <t>7Z03I7</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>7QPP1E</t>
+          <t>9TC0R3</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>6YM9QL</t>
+          <t>IUD5J0</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>D2CHC1</t>
+          <t>0JVXK0</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>HLUWIJ</t>
+          <t>O3VDGR</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>PDEF75</t>
+          <t>RI5BPE</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>YM6165</t>
+          <t>U5T21S</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>HA1ZL6</t>
+          <t>BJFSHV</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>5JI1S9</t>
+          <t>VFXV34</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>NG0Q3P</t>
+          <t>GZL2UT</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>U93FTX</t>
+          <t>8JXNDA</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>DFY5MG</t>
+          <t>JH3YKM</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2AVSZ5</t>
+          <t>5KCEHH</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>D0QZWP</t>
+          <t>ZOJULA</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>9GVAJ9</t>
+          <t>LSQTUB</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>95KJ9W</t>
+          <t>JQ613H</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>RJQMYQ</t>
+          <t>JNMNY6</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>72J88P</t>
+          <t>08X374</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>B1D9NF</t>
+          <t>OHVJ4F</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>1ZXS8H</t>
+          <t>B6DYF1</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>KJ8HA4</t>
+          <t>5ZP67B</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>0KM8J8</t>
+          <t>RCE3W7</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>6I0KH0</t>
+          <t>Z8IS2Q</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>SWPVX7</t>
+          <t>K01R0F</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>NR5KZX</t>
+          <t>8506TC</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>BQ9MZJ</t>
+          <t>ZP2Q7X</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>DEH3JZ</t>
+          <t>J61WER</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>DZH6OU</t>
+          <t>PHL9HB</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>ONXPAK</t>
+          <t>1ZTDOL</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>DQ1E9K</t>
+          <t>0EHZ60</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>JNGRWI</t>
+          <t>PW1E6T</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>XYP6KH</t>
+          <t>7NA8ZO</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>YH8EFT</t>
+          <t>PRMDQB</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>C7Y6GP</t>
+          <t>UX3DI8</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>QG542X</t>
+          <t>RABMMM</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>7SHFBS</t>
+          <t>WXR1AV</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>LMJXVR</t>
+          <t>RC1BML</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>TWE83J</t>
+          <t>6OBV5H</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>7OYZD5</t>
+          <t>PR5H2A</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>1V1Z3Z</t>
+          <t>7798BM</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>017XOR</t>
+          <t>CF5WKF</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>86FCTX</t>
+          <t>VV1GCE</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>05OHFL</t>
+          <t>5EN80W</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Z35EF8</t>
+          <t>VK9WZ4</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>OJDTZE</t>
+          <t>20VU8V</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>RWFNWD</t>
+          <t>6YNQG5</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>YD643D</t>
+          <t>D9BRFR</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>HEFQ0K</t>
+          <t>8Z208A</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>EYQBQ1</t>
+          <t>5QZCO3</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>8U0LQ9</t>
+          <t>KP6ETU</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>CP11W0</t>
+          <t>YINPRU</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>PWL26T</t>
+          <t>FS8OSU</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>3A1ZVU</t>
+          <t>I6D7UW</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Z5KLRR</t>
+          <t>VL8FBM</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>0FM6PE</t>
+          <t>T6XYXD</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>ACSWOW</t>
+          <t>MJXVBD</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>VYS6M9</t>
+          <t>JOMVEA</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Y6NCF5</t>
+          <t>NR9JW5</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>ABTEW6</t>
+          <t>E4KX9U</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>JKFTJI</t>
+          <t>EFQW2T</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>V6T7RZ</t>
+          <t>88MI1Y</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>KDUE6F</t>
+          <t>MW6G28</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>8QEMR2</t>
+          <t>7PYWZH</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>UQZCNM</t>
+          <t>RE5W4H</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>F7J2BX</t>
+          <t>WLOLVB</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>3KPR6D</t>
+          <t>49PUBT</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>934JIB</t>
+          <t>8UH5PZ</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>CJ168M</t>
+          <t>FJ2QWE</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>S36M2W</t>
+          <t>ONHILM</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>NZQC2J</t>
+          <t>8YNUXC</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>BIFM33</t>
+          <t>Y6G4QH</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>K8I0GV</t>
+          <t>IRXD61</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>YIOPP6</t>
+          <t>EZAB74</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>B95T5M</t>
+          <t>ZTMJIT</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>RKGZ3M</t>
+          <t>57T5LP</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>AIWDAH</t>
+          <t>1A3BE4</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>31Q0CT</t>
+          <t>W6OLVN</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>AWEZ8C</t>
+          <t>JIMC0T</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>YG1QVX</t>
+          <t>ETSF72</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>73SMHW</t>
+          <t>S91SEB</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>5BJXRW</t>
+          <t>224K3A</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>MFE2NK</t>
+          <t>BPE42B</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>OBX5V8</t>
+          <t>YK821M</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>4TS32F</t>
+          <t>821PXW</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>MW7K67</t>
+          <t>WV0D47</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2W4ODE</t>
+          <t>VYDGU4</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>K8TUR4</t>
+          <t>4RX3TF</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>L5MHF9</t>
+          <t>080VM7</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>8TM3T9</t>
+          <t>Q6HW5F</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>6SRZJO</t>
+          <t>DW2GKO</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>R0MCMK</t>
+          <t>YAA1IN</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>IOHJD4</t>
+          <t>KP7QUG</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>PS8G7D</t>
+          <t>HKD9YN</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>ESX6X2</t>
+          <t>BWJA7W</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>0P4O9C</t>
+          <t>LX6B3X</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>INXFYM</t>
+          <t>ZE475B</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>C6ANLY</t>
+          <t>U8908U</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>ZLJQYB</t>
+          <t>6NX9BV</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>3DADD3</t>
+          <t>DW3JXT</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>8JA7X1</t>
+          <t>AJLK8I</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2RD263</t>
+          <t>56T860</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>9JYYE6</t>
+          <t>CNBY1R</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>OEHNKQ</t>
+          <t>V5ERS2</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>IQZKCF</t>
+          <t>GJQCZL</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>BMBGPD</t>
+          <t>TR1DUV</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>LGURDB</t>
+          <t>5COY98</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>KD6L2J</t>
+          <t>ONURRZ</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>1HOE1K</t>
+          <t>WUFG4K</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>WKU2QA</t>
+          <t>N98I2F</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>T60QD1</t>
+          <t>1X6E68</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>ZVXSQR</t>
+          <t>B9CYN8</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>EE4G1D</t>
+          <t>N5VTFT</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>4LLIHI</t>
+          <t>HUHPNB</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>Q0QS1B</t>
+          <t>1X85RA</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>X13O77</t>
+          <t>H71YSD</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>OFFGKB</t>
+          <t>J5C71S</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>0T82VL</t>
+          <t>VJVZFB</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>PZWTGN</t>
+          <t>69RIGJ</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2WBDTR</t>
+          <t>8J915B</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>5GJ95U</t>
+          <t>CYM4DH</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>91S7D3</t>
+          <t>SWZM5D</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>LZGANB</t>
+          <t>BMFS3Q</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>ACSS3S</t>
+          <t>ML8M0N</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>ID4RU3</t>
+          <t>ZQM0ZV</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>AM4E6K</t>
+          <t>7ZFLOT</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>1O18K2</t>
+          <t>FR6H3S</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>9T8C29</t>
+          <t>1AAPR6</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>C04VLN</t>
+          <t>9XEAUT</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>8BMM79</t>
+          <t>UV6NCP</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>8XVO9K</t>
+          <t>Z58WVR</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>CV75HC</t>
+          <t>GWD44R</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>K00QD1</t>
+          <t>F7FT13</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>OSP0WY</t>
+          <t>U0W0YM</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>RZSIP1</t>
+          <t>SZXLGK</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>1VE2MG</t>
+          <t>14EZFN</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>SZFPBA</t>
+          <t>ZJ0PDH</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>DZY37L</t>
+          <t>P542LA</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>28ANS0</t>
+          <t>8EJV29</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>F1C14A</t>
+          <t>EKRD0S</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>D4CBY6</t>
+          <t>84LDA6</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>OJ6NBT</t>
+          <t>GSSZM5</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>7Y9CMG</t>
+          <t>U0VCMD</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>EPR2DH</t>
+          <t>V5DF59</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>HJ6FE9</t>
+          <t>1KKJKX</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>RDXGUA</t>
+          <t>14NUN7</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>60L8UO</t>
+          <t>W2DDF7</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>1NE6RV</t>
+          <t>GUK6BC</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>KS92HR</t>
+          <t>46FK54</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>FDA7RI</t>
+          <t>6VDNMA</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>01IL99</t>
+          <t>5X12S1</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>BKKEZP</t>
+          <t>IU97E9</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>T417FW</t>
+          <t>SUB7ID</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>E6HY3C</t>
+          <t>O5DJXL</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>3R1BYP</t>
+          <t>L7P3TN</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>DZWYIP</t>
+          <t>YBVAI3</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>6ZRUKC</t>
+          <t>GHMGAX</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>D0RKLO</t>
+          <t>J61CPX</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>W00DV6</t>
+          <t>4XWSRC</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>P7OAEH</t>
+          <t>FRTS6J</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>52KYW9</t>
+          <t>BKVRRN</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>8A6B02</t>
+          <t>WWTDEP</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>HQ3BWX</t>
+          <t>C3HLPB</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>SDPLCG</t>
+          <t>8P5NEW</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>GGCAZY</t>
+          <t>4960V8</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>RNCB0W</t>
+          <t>12TF1J</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>GTFWKA</t>
+          <t>TA0R4O</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>Y3JVT5</t>
+          <t>Y294SK</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>LGQNS6</t>
+          <t>L3M2MB</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>0BTXMO</t>
+          <t>Q5DNT9</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>QKXWQO</t>
+          <t>N8O1YI</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>34TA5N</t>
+          <t>FERU5A</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>O90KZX</t>
+          <t>CAHWU9</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>PNJBIO</t>
+          <t>8AS9IU</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>CXQZ8W</t>
+          <t>0IPU2G</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>FEUJCS</t>
+          <t>2C313W</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>7HS6GU</t>
+          <t>H1IAKH</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>DI31AX</t>
+          <t>JFABO7</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>CVQYVZ</t>
+          <t>IOZ16H</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>DWTK6T</t>
+          <t>YCG8ZN</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>QSQFP9</t>
+          <t>TTXC4H</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>VEFFU1</t>
+          <t>D95VRS</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>R3ZG6V</t>
+          <t>9810ST</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>3TH5I2</t>
+          <t>71077U</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>SPVOZV</t>
+          <t>PJGQBX</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>LWNV72</t>
+          <t>CAGAHY</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>E8LE5Q</t>
+          <t>7JDR52</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>4CC9JQ</t>
+          <t>9G8JU6</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>ZE5MS9</t>
+          <t>XGSRDV</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>IW392Y</t>
+          <t>6YFADZ</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>0XNE34</t>
+          <t>WWKADC</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>AD6SQH</t>
+          <t>YIHS7C</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>BQMYS6</t>
+          <t>TU3J4P</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>0LKV1I</t>
+          <t>KCDHN1</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>IEWNA8</t>
+          <t>OY1Q7G</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>9RW1SS</t>
+          <t>IJMK24</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>BW1XXO</t>
+          <t>PMDJDD</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>CUQ3I9</t>
+          <t>E58HLG</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>SHNW01</t>
+          <t>8ABZKV</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>X1REV1</t>
+          <t>WG19X9</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>D8RE8X</t>
+          <t>H572Z8</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>71TZJK</t>
+          <t>DLECCN</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>ZOJX7X</t>
+          <t>NQ66EN</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>ZW7F6K</t>
+          <t>TJ692C</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2B2OUD</t>
+          <t>2SMFJ2</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>T2EC8T</t>
+          <t>56WLII</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>QFFF2R</t>
+          <t>HHT6U7</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>V0JJ6A</t>
+          <t>Y3YBU2</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>MNDGEO</t>
+          <t>MN04HD</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>QQOBLL</t>
+          <t>SHVMU8</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>RRSH9G</t>
+          <t>4AZEOP</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>39XCR9</t>
+          <t>NM61GR</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>BVQAR9</t>
+          <t>9BHJ6T</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>DSI6MD</t>
+          <t>5KJ0BX</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>UZXFRR</t>
+          <t>SH1M24</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>NT1H3N</t>
+          <t>RWBEHV</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>E403MC</t>
+          <t>6IAN5U</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>NAPRFQ</t>
+          <t>ZBHPT9</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>KEZSB8</t>
+          <t>0QTZKT</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>ZMVLH6</t>
+          <t>74WWXO</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>BNX0AL</t>
+          <t>ZJW52U</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>IF9Z3D</t>
+          <t>DOWOTO</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>Z4MZ09</t>
+          <t>8N3EJZ</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>K917S0</t>
+          <t>FG3Z6R</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>MTPEIF</t>
+          <t>675H3P</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>9AC6XP</t>
+          <t>M9II82</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>HJ47YH</t>
+          <t>C7TBP7</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>2DKHLY</t>
+          <t>SKT1DP</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>42MT8Y</t>
+          <t>L2DPE3</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>4GCUJI</t>
+          <t>V5JC8U</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>MGAMAO</t>
+          <t>DS91YF</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>V2OWA4</t>
+          <t>7B3Z9P</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>BWOFE1</t>
+          <t>ZZI484</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>302VDW</t>
+          <t>KTR58B</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>E8MPGC</t>
+          <t>W5E190</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>TN746L</t>
+          <t>R7UCWB</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>GMRFPM</t>
+          <t>V3XGLJ</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>UFKRFD</t>
+          <t>CENCY8</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>RZYFBF</t>
+          <t>J09O3L</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>LODLOM</t>
+          <t>SQF3SI</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>QLHZAH</t>
+          <t>39AOPU</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>Q5PT5W</t>
+          <t>MQ1KXL</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>6MOGUL</t>
+          <t>GH4CHR</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>J0BA1C</t>
+          <t>F5OWDB</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>0ECP01</t>
+          <t>GSKQ6X</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>8XQIAK</t>
+          <t>8KWQY6</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>1H8FWI</t>
+          <t>KFJETV</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>72NFDI</t>
+          <t>RDCLP7</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>C9NXLW</t>
+          <t>Q7RZF0</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>0WSCNU</t>
+          <t>66SN2N</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>VDC8KP</t>
+          <t>P1PXKZ</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>EL41WV</t>
+          <t>M48HBO</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>AGJSPC</t>
+          <t>4LPMT3</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>745GJQ</t>
+          <t>WXLANS</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>HZSRSG</t>
+          <t>CIRY0R</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>GVXB6F</t>
+          <t>KA3QNS</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>NIFWOU</t>
+          <t>KAZBWE</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>IHYTP4</t>
+          <t>1EDIA1</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>BPM2W5</t>
+          <t>CE02MR</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>IARC4H</t>
+          <t>07Q2QS</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>WT6V98</t>
+          <t>EVQI39</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>LAEDJS</t>
+          <t>HG4R48</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>8NNOJ7</t>
+          <t>04HSAM</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>XBU0MM</t>
+          <t>ETSZ1I</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>06C3MG</t>
+          <t>OSTELY</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>6RBCXL</t>
+          <t>KQ6YKK</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>JJU9VH</t>
+          <t>J1K33M</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>M3PURS</t>
+          <t>37TNEQ</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>AY5IPV</t>
+          <t>FPPP5V</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>I6SI3A</t>
+          <t>H20OQ1</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>RI4WHS</t>
+          <t>ZCBTHZ</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>U8YWVB</t>
+          <t>BBM0W5</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>Z4KJ5R</t>
+          <t>I3VS2A</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>C0J78T</t>
+          <t>8KJMOT</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>X8JUML</t>
+          <t>3J6SEW</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>IIHJC7</t>
+          <t>8YU4FC</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>AFU36W</t>
+          <t>QISL7X</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>2X8WVM</t>
+          <t>PVHDHT</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>FMP9IU</t>
+          <t>8Z3UOT</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>THQULT</t>
+          <t>5J41ZF</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>MZLLVL</t>
+          <t>IU2SQ9</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>P8PJ5Y</t>
+          <t>YF9GGM</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>MCGOX8</t>
+          <t>DUTH74</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>QWYSVM</t>
+          <t>TU2S1R</t>
         </is>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>B744RW</t>
+          <t>2RTJ1Q</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>QPBUT1</t>
+          <t>ADH5LU</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>UNX8PD</t>
+          <t>DZCVVL</t>
         </is>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>6FMX19</t>
+          <t>P6B1PH</t>
         </is>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>LC98T7</t>
+          <t>XHVZIN</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>7O32BC</t>
+          <t>U813R0</t>
         </is>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>M6MYZB</t>
+          <t>5XHO3G</t>
         </is>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>5UU3D1</t>
+          <t>NCS043</t>
         </is>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>1C0RZM</t>
+          <t>1EVTX9</t>
         </is>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>CKB9GU</t>
+          <t>B4HHDD</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
         <is>
-          <t>22NW1E</t>
+          <t>Z7T423</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
         <is>
-          <t>W240CP</t>
+          <t>PXYHCT</t>
         </is>
       </c>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
         <is>
-          <t>OINHAO</t>
+          <t>1NE8ZS</t>
         </is>
       </c>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>BYNHC7</t>
+          <t>VZQ65L</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>MWRR06</t>
+          <t>NW3LDQ</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
-          <t>J49LKR</t>
+          <t>JRIH0A</t>
         </is>
       </c>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
         <is>
-          <t>6A8PMM</t>
+          <t>RWB8AO</t>
         </is>
       </c>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
         <is>
-          <t>RW7NT1</t>
+          <t>K4HKY3</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
         <is>
-          <t>TCDKQW</t>
+          <t>PJS72E</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>FMF0UB</t>
+          <t>GAAQBD</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>9GM98Z</t>
+          <t>0U613K</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>40XXKR</t>
+          <t>CJOSR2</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>E5OI4R</t>
+          <t>HPLOWZ</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>ZSREU9</t>
+          <t>VNNK47</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>XEKHPK</t>
+          <t>WFGCY3</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>K5QC8D</t>
+          <t>TCHWTX</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
         <is>
-          <t>599I0F</t>
+          <t>XCHSRK</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
         <is>
-          <t>1CVZ45</t>
+          <t>3ZJSMB</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>YIFCR1</t>
+          <t>R8O50E</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
         <is>
-          <t>8LRHQN</t>
+          <t>3RD8MH</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>I6428B</t>
+          <t>PX8PHL</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>FIZB9B</t>
+          <t>XJFNIE</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>NJF8MN</t>
+          <t>DH8GWL</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>8VJ7WN</t>
+          <t>OM8DFF</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>PINNZ6</t>
+          <t>2K3XZ7</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>MHQRD8</t>
+          <t>22D9ET</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>9V37G2</t>
+          <t>Z2UQ8R</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>ZDMSZC</t>
+          <t>OQVDWH</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>9G8WYE</t>
+          <t>PDLNPV</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>F9YL8M</t>
+          <t>RPFJHP</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>BVVI6B</t>
+          <t>OL9QQS</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>8NQK09</t>
+          <t>LHJTY1</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>XJQ332</t>
+          <t>YTTK4F</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>XUWM7A</t>
+          <t>WZWULN</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>1HPHB5</t>
+          <t>4HX9YI</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>MQEX79</t>
+          <t>RQRT7A</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>WKYNW7</t>
+          <t>TY898F</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
         <is>
-          <t>BWQMUH</t>
+          <t>HJ9KVC</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
         <is>
-          <t>Y6BW93</t>
+          <t>6T8GIG</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>Z2MOLR</t>
+          <t>2676AH</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
-          <t>P4OGN6</t>
+          <t>R0OEFC</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>2YOE1U</t>
+          <t>3NOR4X</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>MCS1TF</t>
+          <t>VNQNOC</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>CGCOR5</t>
+          <t>BT1QLD</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>T4BOH2</t>
+          <t>9YF8VR</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>PTZGUV</t>
+          <t>2CLWJQ</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
         <is>
-          <t>ETC9V4</t>
+          <t>KDO9VY</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>RWU6XO</t>
+          <t>SVCJH1</t>
         </is>
       </c>
     </row>
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
-          <t>BBFLX0</t>
+          <t>U5HF06</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
         <is>
-          <t>9BFJIZ</t>
+          <t>PSTK94</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
         <is>
-          <t>XHKHBU</t>
+          <t>JF0CUX</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t>2PMVLQ</t>
+          <t>1H05QY</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>63WVFY</t>
+          <t>4SER5H</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="A431" t="inlineStr">
         <is>
-          <t>ZO49G6</t>
+          <t>NAXXEC</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>87SX3C</t>
+          <t>12OIOS</t>
         </is>
       </c>
     </row>
     <row r="433">
       <c r="A433" t="inlineStr">
         <is>
-          <t>XZ5YTG</t>
+          <t>03BOFT</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" t="inlineStr">
         <is>
-          <t>PHA5U8</t>
+          <t>V80FNE</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t>GXQBRP</t>
+          <t>FX330K</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="A436" t="inlineStr">
         <is>
-          <t>W4YP61</t>
+          <t>V9Z250</t>
         </is>
       </c>
     </row>
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t>JRLQTC</t>
+          <t>8EBXOB</t>
         </is>
       </c>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
         <is>
-          <t>XP81L1</t>
+          <t>LJ2AHG</t>
         </is>
       </c>
     </row>
     <row r="439">
       <c r="A439" t="inlineStr">
         <is>
-          <t>ZD2ZJI</t>
+          <t>4E64I5</t>
         </is>
       </c>
     </row>
     <row r="440">
       <c r="A440" t="inlineStr">
         <is>
-          <t>AAURSO</t>
+          <t>EY09PB</t>
         </is>
       </c>
     </row>
     <row r="441">
       <c r="A441" t="inlineStr">
         <is>
-          <t>42VUV4</t>
+          <t>DR54LK</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>XOLNXK</t>
+          <t>GFWMSB</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>GOZ8X3</t>
+          <t>T5BI0C</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="A444" t="inlineStr">
         <is>
-          <t>U1LXCK</t>
+          <t>YGH519</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="A445" t="inlineStr">
         <is>
-          <t>QY8CPD</t>
+          <t>1TM2VY</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
         <is>
-          <t>F7HF8Y</t>
+          <t>9G31CL</t>
         </is>
       </c>
     </row>
     <row r="447">
       <c r="A447" t="inlineStr">
         <is>
-          <t>PY9WEV</t>
+          <t>PGZ2EY</t>
         </is>
       </c>
     </row>
     <row r="448">
       <c r="A448" t="inlineStr">
         <is>
-          <t>BIN1K2</t>
+          <t>I3W4CS</t>
         </is>
       </c>
     </row>
     <row r="449">
       <c r="A449" t="inlineStr">
         <is>
-          <t>TYDPFJ</t>
+          <t>7NZESG</t>
         </is>
       </c>
     </row>
     <row r="450">
       <c r="A450" t="inlineStr">
         <is>
-          <t>FBUET8</t>
+          <t>U6XOFY</t>
         </is>
       </c>
     </row>
     <row r="451">
       <c r="A451" t="inlineStr">
         <is>
-          <t>ZV2Z0H</t>
+          <t>DC00S2</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
         <is>
-          <t>TF6IQY</t>
+          <t>2CM4VN</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
         <is>
-          <t>UOWAB6</t>
+          <t>1ZOVD1</t>
         </is>
       </c>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr">
         <is>
-          <t>MFG22K</t>
+          <t>69LRIK</t>
         </is>
       </c>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
         <is>
-          <t>X9MP9Q</t>
+          <t>M5EO9A</t>
         </is>
       </c>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
         <is>
-          <t>CRXBWV</t>
+          <t>H8PU15</t>
         </is>
       </c>
     </row>
     <row r="457">
       <c r="A457" t="inlineStr">
         <is>
-          <t>J7AOAS</t>
+          <t>ZPCTQV</t>
         </is>
       </c>
     </row>
     <row r="458">
       <c r="A458" t="inlineStr">
         <is>
-          <t>3P0NUV</t>
+          <t>AEJNU6</t>
         </is>
       </c>
     </row>
     <row r="459">
       <c r="A459" t="inlineStr">
         <is>
-          <t>1CVB2R</t>
+          <t>INWUH6</t>
         </is>
       </c>
     </row>
     <row r="460">
       <c r="A460" t="inlineStr">
         <is>
-          <t>IJLR83</t>
+          <t>YX0QMZ</t>
         </is>
       </c>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
         <is>
-          <t>ICOOYE</t>
+          <t>E4PDAN</t>
         </is>
       </c>
     </row>
     <row r="462">
       <c r="A462" t="inlineStr">
         <is>
-          <t>P7J2B8</t>
+          <t>02AAJC</t>
         </is>
       </c>
     </row>
     <row r="463">
       <c r="A463" t="inlineStr">
         <is>
-          <t>O5WIOA</t>
+          <t>HU23M6</t>
         </is>
       </c>
     </row>
     <row r="464">
       <c r="A464" t="inlineStr">
         <is>
-          <t>M9HWI5</t>
+          <t>G7JYCG</t>
         </is>
       </c>
     </row>
     <row r="465">
       <c r="A465" t="inlineStr">
         <is>
-          <t>55IYUO</t>
+          <t>BKTNUP</t>
         </is>
       </c>
     </row>
     <row r="466">
       <c r="A466" t="inlineStr">
         <is>
-          <t>C3Q8YG</t>
+          <t>UY1O76</t>
         </is>
       </c>
     </row>
     <row r="467">
       <c r="A467" t="inlineStr">
         <is>
-          <t>E1FQ19</t>
+          <t>K5XDNB</t>
         </is>
       </c>
     </row>
     <row r="468">
       <c r="A468" t="inlineStr">
         <is>
-          <t>B190VE</t>
+          <t>DP49B7</t>
         </is>
       </c>
     </row>
     <row r="469">
       <c r="A469" t="inlineStr">
         <is>
-          <t>A2DU0H</t>
+          <t>N15ES5</t>
         </is>
       </c>
     </row>
     <row r="470">
       <c r="A470" t="inlineStr">
         <is>
-          <t>QE56OM</t>
+          <t>BGTT2Q</t>
         </is>
       </c>
     </row>
     <row r="471">
       <c r="A471" t="inlineStr">
         <is>
-          <t>4V74Z3</t>
+          <t>T50W8Q</t>
         </is>
       </c>
     </row>
     <row r="472">
       <c r="A472" t="inlineStr">
         <is>
-          <t>CXHB9B</t>
+          <t>3MFWGC</t>
         </is>
       </c>
     </row>
     <row r="473">
       <c r="A473" t="inlineStr">
         <is>
-          <t>DWYJQL</t>
+          <t>69LZTS</t>
         </is>
       </c>
     </row>
     <row r="474">
       <c r="A474" t="inlineStr">
         <is>
-          <t>R20X2O</t>
+          <t>KGT4CU</t>
         </is>
       </c>
     </row>
     <row r="475">
       <c r="A475" t="inlineStr">
         <is>
-          <t>KKSGGA</t>
+          <t>MZAG52</t>
         </is>
       </c>
     </row>
     <row r="476">
       <c r="A476" t="inlineStr">
         <is>
-          <t>OQRTOT</t>
+          <t>7H7XJP</t>
         </is>
       </c>
     </row>
     <row r="477">
       <c r="A477" t="inlineStr">
         <is>
-          <t>DF2AFN</t>
+          <t>BNDADB</t>
         </is>
       </c>
     </row>
     <row r="478">
       <c r="A478" t="inlineStr">
         <is>
-          <t>RBEAGF</t>
+          <t>S9UHRF</t>
         </is>
       </c>
     </row>
     <row r="479">
       <c r="A479" t="inlineStr">
         <is>
-          <t>ICNITD</t>
+          <t>N8OHB3</t>
         </is>
       </c>
     </row>
     <row r="480">
       <c r="A480" t="inlineStr">
         <is>
-          <t>DJ4XFB</t>
+          <t>G0ZURD</t>
         </is>
       </c>
     </row>
     <row r="481">
       <c r="A481" t="inlineStr">
         <is>
-          <t>2F45JD</t>
+          <t>QZSBMG</t>
         </is>
       </c>
     </row>
     <row r="482">
       <c r="A482" t="inlineStr">
         <is>
-          <t>ZOS4AK</t>
+          <t>O7VPLY</t>
         </is>
       </c>
     </row>
     <row r="483">
       <c r="A483" t="inlineStr">
         <is>
-          <t>QWNZLK</t>
+          <t>0CM2MM</t>
         </is>
       </c>
     </row>
     <row r="484">
       <c r="A484" t="inlineStr">
         <is>
-          <t>KD56S7</t>
+          <t>5Q0UOH</t>
         </is>
       </c>
     </row>
     <row r="485">
       <c r="A485" t="inlineStr">
         <is>
-          <t>CYLQXT</t>
+          <t>Y0IO5K</t>
         </is>
       </c>
     </row>
     <row r="486">
       <c r="A486" t="inlineStr">
         <is>
-          <t>06EQAM</t>
+          <t>UGE5R7</t>
         </is>
       </c>
     </row>
     <row r="487">
       <c r="A487" t="inlineStr">
         <is>
-          <t>HQITHJ</t>
+          <t>DDHEOH</t>
         </is>
       </c>
     </row>
     <row r="488">
       <c r="A488" t="inlineStr">
         <is>
-          <t>HCMBDS</t>
+          <t>N3ILUZ</t>
         </is>
       </c>
     </row>
     <row r="489">
       <c r="A489" t="inlineStr">
         <is>
-          <t>FVOAH5</t>
+          <t>D0PCAO</t>
         </is>
       </c>
     </row>
     <row r="490">
       <c r="A490" t="inlineStr">
         <is>
-          <t>9C1HD1</t>
+          <t>J3T1Z0</t>
         </is>
       </c>
     </row>
     <row r="491">
       <c r="A491" t="inlineStr">
         <is>
-          <t>0RXO1Q</t>
+          <t>NPJ9TI</t>
         </is>
       </c>
     </row>
     <row r="492">
       <c r="A492" t="inlineStr">
         <is>
-          <t>59AY8T</t>
+          <t>TWKRPB</t>
         </is>
       </c>
     </row>
     <row r="493">
       <c r="A493" t="inlineStr">
         <is>
-          <t>UGBG3Q</t>
+          <t>I7N3R2</t>
         </is>
       </c>
     </row>
     <row r="494">
       <c r="A494" t="inlineStr">
         <is>
-          <t>MZMOF2</t>
+          <t>56MZZ4</t>
         </is>
       </c>
     </row>
     <row r="495">
       <c r="A495" t="inlineStr">
         <is>
-          <t>Z35LVP</t>
+          <t>45WNB7</t>
         </is>
       </c>
     </row>
     <row r="496">
       <c r="A496" t="inlineStr">
         <is>
-          <t>I4IXPX</t>
+          <t>S2VOHZ</t>
         </is>
       </c>
     </row>
     <row r="497">
       <c r="A497" t="inlineStr">
         <is>
-          <t>BQX8ZX</t>
+          <t>W1MFOJ</t>
         </is>
       </c>
     </row>
     <row r="498">
       <c r="A498" t="inlineStr">
         <is>
-          <t>4FTJGQ</t>
+          <t>GEKXZN</t>
         </is>
       </c>
     </row>
     <row r="499">
       <c r="A499" t="inlineStr">
         <is>
-          <t>CSD0BW</t>
+          <t>IXEP4C</t>
         </is>
       </c>
     </row>
     <row r="500">
       <c r="A500" t="inlineStr">
         <is>
-          <t>I4VLH4</t>
+          <t>0WHIED</t>
         </is>
       </c>
     </row>
     <row r="501">
       <c r="A501" t="inlineStr">
         <is>
-          <t>SCEKF8</t>
+          <t>QY4C80</t>
         </is>
       </c>
     </row>

</xml_diff>